<commit_message>
add second expense page and update README
</commit_message>
<xml_diff>
--- a/Mock data.xlsx
+++ b/Mock data.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Data_projects\Bank\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\Data_projects\bank_statement_vis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{977D0D11-092A-4E1F-9650-359F1ABE8D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFEA2B1-339D-425F-B737-9A7B7DA9110A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{8726AD55-5608-4A15-AFBE-AC59A45A8531}"/>
   </bookViews>
   <sheets>
-    <sheet name="Mock data" sheetId="1" r:id="rId1"/>
+    <sheet name="Essential" sheetId="3" r:id="rId1"/>
+    <sheet name="Mock data" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10531" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10553" uniqueCount="93">
   <si>
     <t>Date</t>
   </si>
@@ -290,6 +291,15 @@
   </si>
   <si>
     <t>Aldi</t>
+  </si>
+  <si>
+    <t>Essential</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
@@ -773,10 +783,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1151,6 +1164,107 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57B36BB0-19E8-4B76-B1BF-1D410313AD83}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C466DAC0-2D83-4914-8C75-40C3FE32249C}">
   <dimension ref="A1:G3509"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>